<commit_message>
feat: implement carousel, pdf font update, and new materials form layout
</commit_message>
<xml_diff>
--- a/Fise de laborator.xlsx
+++ b/Fise de laborator.xlsx
@@ -5,16 +5,19 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7844f1ebed51f8b9/Documente/ClaSerDent Technology/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/eaed5ce4aff0af09/Desktop/fisa laborator/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="14_{4EDD655F-83B9-464E-B2B8-069FE538CD12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{248E16C3-F6FF-4687-9DD9-62F209BDCA2A}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D6312EDC-FA11-4532-8F9A-1164E5950395}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A9C541A9-953D-4AA7-80AC-9AB554C8C448}"/>
+    <workbookView xWindow="10650" yWindow="3060" windowWidth="13290" windowHeight="11295" xr2:uid="{A9C541A9-953D-4AA7-80AC-9AB554C8C448}"/>
   </bookViews>
   <sheets>
     <sheet name="Foaie1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Foaie1!$A$1:$J$47</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -36,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
   <si>
     <t>Dl./Dna. Doctor:</t>
   </si>
@@ -47,33 +50,9 @@
     <t>Culoare:</t>
   </si>
   <si>
-    <t>La colet:</t>
-  </si>
-  <si>
     <t>Termen de livrare:</t>
   </si>
   <si>
-    <t>Material:</t>
-  </si>
-  <si>
-    <t>Zirconiu</t>
-  </si>
-  <si>
-    <t>Aur</t>
-  </si>
-  <si>
-    <t>CrCo</t>
-  </si>
-  <si>
-    <t>Cr.Ni</t>
-  </si>
-  <si>
-    <t>Titan</t>
-  </si>
-  <si>
-    <t>Forma dinţilor:</t>
-  </si>
-  <si>
     <t>Schiţa pentru culoare:</t>
   </si>
   <si>
@@ -92,29 +71,68 @@
     <t xml:space="preserve">                                  De asemenea, ea reprezintă şi confirmarea comenzii şi afară de aceasta nu există o altă confirmare</t>
   </si>
   <si>
-    <t xml:space="preserve">                  Laborator de Tehnica Dentara </t>
-  </si>
-  <si>
-    <t xml:space="preserve">                  ClaSerDent Technology S.R.L.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">            Calea Clujului Nr. 231 C, Oradea, Bihor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">                               Cui: 47130210</t>
-  </si>
-  <si>
-    <t xml:space="preserve">             Email: claserdenttechnology@gmail.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">                           Telefon: 0773 783 114</t>
+    <t>Cervical:</t>
+  </si>
+  <si>
+    <t>Tip lucrare:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">                             Cui: 47130210</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Monolitici</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> PMMA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  DCR CrCo</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> MC Basic</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  MC Pers.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Zr. + e.max</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Scheletata</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Fateta dent.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  DCR Zr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Onlay/Inlay</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  All On X</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         Email: claserdenttechnology@gmail.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">                      Telefon: 0773 783 114</t>
+  </si>
+  <si>
+    <t xml:space="preserve">          Calea Clujului Nr. 231 C, Oradea, Bihor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">               Laborator de Tehnica Dentara </t>
+  </si>
+  <si>
+    <t xml:space="preserve">                ClaSerDent Technology S.R.L.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -159,6 +177,20 @@
       <family val="1"/>
       <charset val="238"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="8"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -168,7 +200,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="15">
+  <borders count="20">
     <border>
       <left/>
       <right/>
@@ -196,19 +228,6 @@
     </border>
     <border>
       <left/>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
       <right/>
       <top style="thin">
         <color auto="1"/>
@@ -281,26 +300,6 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right style="medium">
-        <color auto="1"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="medium">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="medium">
         <color auto="1"/>
       </left>
@@ -313,13 +312,129 @@
     </border>
     <border>
       <left/>
+      <right style="dashed">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="dashed">
+        <color auto="1"/>
+      </left>
+      <right style="dashed">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="dashed">
+        <color auto="1"/>
+      </left>
       <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="dashed">
         <color auto="1"/>
       </right>
       <top style="thin">
         <color auto="1"/>
       </top>
       <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="dashed">
+        <color auto="1"/>
+      </left>
+      <right style="dashed">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="dashed">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="dashed">
+        <color auto="1"/>
+      </left>
+      <right style="dashed">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="dashed">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="dashed">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
         <color auto="1"/>
       </bottom>
       <diagonal/>
@@ -328,51 +443,88 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -395,15 +547,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>193962</xdr:colOff>
-      <xdr:row>11</xdr:row>
-      <xdr:rowOff>106507</xdr:rowOff>
+      <xdr:colOff>145646</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>182431</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>515681</xdr:colOff>
-      <xdr:row>19</xdr:row>
-      <xdr:rowOff>240723</xdr:rowOff>
+      <xdr:colOff>407177</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>109581</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -432,8 +584,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="193962" y="2834121"/>
-          <a:ext cx="3309105" cy="1398443"/>
+          <a:off x="145646" y="2184061"/>
+          <a:ext cx="3312292" cy="1404216"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -445,15 +597,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>185305</xdr:colOff>
+      <xdr:colOff>109382</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>309130</xdr:rowOff>
+      <xdr:rowOff>74456</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>428626</xdr:colOff>
-      <xdr:row>9</xdr:row>
-      <xdr:rowOff>65337</xdr:rowOff>
+      <xdr:colOff>292515</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>23923</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -482,8 +634,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="185305" y="1149062"/>
-          <a:ext cx="3230707" cy="1254230"/>
+          <a:off x="109382" y="564510"/>
+          <a:ext cx="3233894" cy="1267783"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -495,15 +647,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>162791</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>181842</xdr:rowOff>
+      <xdr:colOff>141257</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>38649</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>400916</xdr:colOff>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>1000034</xdr:colOff>
       <xdr:row>5</xdr:row>
-      <xdr:rowOff>85727</xdr:rowOff>
+      <xdr:rowOff>131050</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -531,58 +683,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="3799609" y="476251"/>
-          <a:ext cx="2662671" cy="830408"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>75468</xdr:colOff>
-      <xdr:row>20</xdr:row>
-      <xdr:rowOff>96783</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>492829</xdr:colOff>
-      <xdr:row>20</xdr:row>
-      <xdr:rowOff>278552</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="17" name="Imagine 16">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DF6404BC-5217-EC8C-67AD-E21216B15F30}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4" cstate="print">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="5530695" y="3872147"/>
-          <a:ext cx="1023498" cy="181769"/>
+          <a:off x="3778075" y="527269"/>
+          <a:ext cx="2695741" cy="828424"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -594,13 +696,13 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>38237</xdr:colOff>
+      <xdr:colOff>615642</xdr:colOff>
       <xdr:row>22</xdr:row>
       <xdr:rowOff>39837</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>209687</xdr:colOff>
+      <xdr:colOff>787092</xdr:colOff>
       <xdr:row>22</xdr:row>
       <xdr:rowOff>207300</xdr:rowOff>
     </xdr:to>
@@ -618,7 +720,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5" cstate="print">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4" cstate="print">
           <a:extLst>
             <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
               <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
@@ -631,57 +733,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm flipV="1">
-          <a:off x="601078" y="4568542"/>
-          <a:ext cx="171450" cy="167463"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>62083</xdr:colOff>
-      <xdr:row>22</xdr:row>
-      <xdr:rowOff>41843</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>233533</xdr:colOff>
-      <xdr:row>22</xdr:row>
-      <xdr:rowOff>209306</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="20" name="Imagine 19">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{793EE7F1-ECD6-4527-A13D-066D679A5F48}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5" cstate="print">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm flipV="1">
-          <a:off x="1360947" y="4570548"/>
+          <a:off x="1473366" y="4494315"/>
           <a:ext cx="171450" cy="167463"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -694,22 +746,22 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>45794</xdr:colOff>
-      <xdr:row>22</xdr:row>
-      <xdr:rowOff>50552</xdr:rowOff>
+      <xdr:colOff>188751</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>48804</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>217244</xdr:colOff>
-      <xdr:row>22</xdr:row>
-      <xdr:rowOff>218015</xdr:rowOff>
+      <xdr:colOff>360201</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>216267</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="21" name="Imagine 20">
+        <xdr:cNvPr id="22" name="Imagine 21">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1CBAA6AD-4D80-49CF-B92A-7CADAB3FA8B8}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C39F5E9C-956B-49FA-BA78-F71341E7E1B4}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -718,7 +770,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5" cstate="print">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4" cstate="print">
           <a:extLst>
             <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
               <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
@@ -731,57 +783,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm flipV="1">
-          <a:off x="1907499" y="4579257"/>
-          <a:ext cx="171450" cy="167463"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>29113</xdr:colOff>
-      <xdr:row>22</xdr:row>
-      <xdr:rowOff>37550</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>200563</xdr:colOff>
-      <xdr:row>22</xdr:row>
-      <xdr:rowOff>205013</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="22" name="Imagine 21">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C39F5E9C-956B-49FA-BA78-F71341E7E1B4}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5" cstate="print">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm flipV="1">
-          <a:off x="2436340" y="4566255"/>
+          <a:off x="2392296" y="4247386"/>
           <a:ext cx="171450" cy="167463"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -794,15 +796,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>32141</xdr:colOff>
+      <xdr:colOff>381343</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>30893</xdr:rowOff>
+      <xdr:rowOff>78725</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>203591</xdr:colOff>
+      <xdr:colOff>552793</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>198356</xdr:rowOff>
+      <xdr:rowOff>246188</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -818,7 +820,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5" cstate="print">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4" cstate="print">
           <a:extLst>
             <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
               <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
@@ -831,7 +833,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm flipV="1">
-          <a:off x="3071482" y="4559598"/>
+          <a:off x="3428395" y="4533203"/>
           <a:ext cx="171450" cy="167463"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -844,15 +846,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>60614</xdr:colOff>
-      <xdr:row>25</xdr:row>
-      <xdr:rowOff>60615</xdr:rowOff>
+      <xdr:colOff>67518</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>45760</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>606826</xdr:colOff>
-      <xdr:row>38</xdr:row>
-      <xdr:rowOff>173182</xdr:rowOff>
+      <xdr:colOff>377691</xdr:colOff>
+      <xdr:row>39</xdr:row>
+      <xdr:rowOff>30793</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -868,7 +870,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5">
           <a:extLst>
             <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
               <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
@@ -881,8 +883,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="60614" y="5221433"/>
-          <a:ext cx="3533598" cy="2589067"/>
+          <a:off x="67518" y="5457064"/>
+          <a:ext cx="3360934" cy="2497425"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -891,6 +893,381 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>617675</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>38669</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>789125</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>206132</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="Imagine 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4E2FF98D-7BCF-4279-BA93-9E02F6A67874}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm flipV="1">
+          <a:off x="1475399" y="4237251"/>
+          <a:ext cx="171450" cy="167463"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>187584</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>51044</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>359034</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>218507</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="8" name="Imagine 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AC34BCCA-9B53-4624-BB12-DC6C40822ECC}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm flipV="1">
+          <a:off x="2391129" y="4505522"/>
+          <a:ext cx="171450" cy="167463"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>388439</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>42147</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>559889</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>209610</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="9" name="Imagine 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9EE46D5F-F15E-4560-9CE6-0851F02510E1}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm flipV="1">
+          <a:off x="3435491" y="4240729"/>
+          <a:ext cx="171450" cy="167463"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>188751</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>77237</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="171450" cy="167463"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Imagine 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{61492690-0FEA-4E6A-A950-4CC4996C37B4}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm flipV="1">
+          <a:off x="2392296" y="3953580"/>
+          <a:ext cx="171450" cy="167463"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>613819</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>87266</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="171450" cy="167463"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Imagine 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D264D45B-D842-4F0E-BBD0-AD9630693806}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm flipV="1">
+          <a:off x="1471543" y="3963609"/>
+          <a:ext cx="171450" cy="167463"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>388439</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>70580</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="171450" cy="167463"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Imagine 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7FBF446D-CFED-4C71-843F-EFD0AD058243}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm flipV="1">
+          <a:off x="3435491" y="3946923"/>
+          <a:ext cx="171450" cy="167463"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>652938</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>44290</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="171450" cy="167463"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="10" name="Imagine 9">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4773CE54-D40A-492A-99D4-B0A36668238D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm flipV="1">
+          <a:off x="652938" y="4242872"/>
+          <a:ext cx="171450" cy="167463"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>644074</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>77747</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="171450" cy="167463"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="12" name="Imagine 11">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F03534BB-CB44-4D6D-AF75-5CD6E8943FB1}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm flipV="1">
+          <a:off x="644074" y="4532225"/>
+          <a:ext cx="171450" cy="167463"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -1194,95 +1571,103 @@
   <dimension ref="A1:K47"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.42578125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="11" style="1" customWidth="1"/>
-    <col min="3" max="3" width="8.42578125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="8.140625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="8.7109375" style="1" customWidth="1"/>
-    <col min="6" max="6" width="9.7109375" style="1" customWidth="1"/>
-    <col min="7" max="10" width="9.140625" style="1"/>
-    <col min="11" max="11" width="8.5703125" style="1" customWidth="1"/>
+    <col min="1" max="1" width="12.85546875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="12.42578125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="7.7109375" style="1" customWidth="1"/>
+    <col min="4" max="4" width="6" style="1" customWidth="1"/>
+    <col min="5" max="5" width="6.7109375" style="1" customWidth="1"/>
+    <col min="6" max="6" width="8.85546875" style="1" customWidth="1"/>
+    <col min="7" max="9" width="9.140625" style="1"/>
+    <col min="10" max="10" width="16.5703125" style="1" customWidth="1"/>
+    <col min="11" max="11" width="1.42578125" style="1" customWidth="1"/>
     <col min="12" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="D1" s="21" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" ht="27.75" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:10" ht="23.25" x14ac:dyDescent="0.35">
+      <c r="D1" s="14" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" ht="27.75" x14ac:dyDescent="0.4">
       <c r="A3" s="2"/>
       <c r="G3" s="3"/>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="G4" s="3"/>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="F5" s="11"/>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="F6" s="11"/>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="F7" s="11"/>
-      <c r="G7" s="25" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="F8" s="11"/>
-      <c r="G8" s="25" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="F9" s="11"/>
-      <c r="G9" s="1" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="F10" s="11"/>
-      <c r="G10" s="1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="F11" s="11"/>
-      <c r="G11" s="1" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="F12" s="11"/>
-      <c r="G12" s="1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" ht="5.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="F13" s="11"/>
-      <c r="G13" s="5"/>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="G5" s="3"/>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="G6" s="3"/>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="G7" s="24" t="s">
+        <v>27</v>
+      </c>
+      <c r="H7" s="25"/>
+      <c r="I7" s="25"/>
+      <c r="J7" s="25"/>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="G8" s="24" t="s">
+        <v>28</v>
+      </c>
+      <c r="H8" s="25"/>
+      <c r="I8" s="25"/>
+      <c r="J8" s="25"/>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="G9" s="26" t="s">
+        <v>12</v>
+      </c>
+      <c r="H9" s="27"/>
+      <c r="I9" s="27"/>
+      <c r="J9" s="27"/>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="G10" s="26" t="s">
+        <v>26</v>
+      </c>
+      <c r="H10" s="27"/>
+      <c r="I10" s="27"/>
+      <c r="J10" s="27"/>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="G11" s="26" t="s">
+        <v>24</v>
+      </c>
+      <c r="H11" s="27"/>
+      <c r="I11" s="27"/>
+      <c r="J11" s="27"/>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="G12" s="26" t="s">
+        <v>25</v>
+      </c>
+      <c r="H12" s="27"/>
+      <c r="I12" s="27"/>
+      <c r="J12" s="27"/>
+    </row>
+    <row r="13" spans="1:10" ht="5.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G13" s="4"/>
       <c r="H13" s="5"/>
       <c r="I13" s="5"/>
       <c r="J13" s="5"/>
-      <c r="K13" s="5"/>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="F14" s="11"/>
-      <c r="G14" s="7" t="s">
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="G14" s="6" t="s">
         <v>0</v>
       </c>
       <c r="H14" s="7"/>
       <c r="I14" s="7"/>
       <c r="J14" s="7"/>
-      <c r="K14" s="7"/>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="G15" s="3"/>
     </row>
-    <row r="16" spans="1:11" ht="9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" ht="9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="G16" s="3"/>
-      <c r="K16" s="5"/>
     </row>
     <row r="17" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="G17" s="6" t="s">
@@ -1291,114 +1676,144 @@
       <c r="H17" s="7"/>
       <c r="I17" s="7"/>
       <c r="J17" s="7"/>
-      <c r="K17" s="7"/>
     </row>
     <row r="18" spans="1:11" ht="6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="G18" s="3"/>
     </row>
     <row r="19" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G19" s="4"/>
-      <c r="H19" s="5"/>
-      <c r="I19" s="5"/>
-      <c r="J19" s="5"/>
-      <c r="K19" s="5"/>
-    </row>
-    <row r="20" spans="1:11" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G19" s="3"/>
+    </row>
+    <row r="20" spans="1:11" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="G20" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="H20" s="5"/>
-      <c r="I20" s="9"/>
-      <c r="J20" s="10" t="s">
+      <c r="H20" s="9"/>
+      <c r="I20" s="29" t="s">
+        <v>10</v>
+      </c>
+      <c r="J20" s="29"/>
+      <c r="K20" s="30"/>
+    </row>
+    <row r="21" spans="1:11" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="18" t="s">
+        <v>11</v>
+      </c>
+      <c r="B21" s="19" t="s">
+        <v>16</v>
+      </c>
+      <c r="C21" s="35" t="s">
+        <v>17</v>
+      </c>
+      <c r="D21" s="35"/>
+      <c r="E21" s="35" t="s">
+        <v>18</v>
+      </c>
+      <c r="F21" s="36"/>
+      <c r="G21" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="K20" s="5"/>
-    </row>
-    <row r="21" spans="1:11" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="F21" s="11"/>
-      <c r="G21" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="H21" s="13"/>
-      <c r="I21" s="14"/>
-      <c r="J21" s="14"/>
-      <c r="K21" s="14"/>
-    </row>
-    <row r="22" spans="1:11" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="F22" s="11"/>
-      <c r="G22" s="15" t="s">
+      <c r="I21" s="15"/>
+      <c r="J21" s="15"/>
+      <c r="K21" s="15"/>
+    </row>
+    <row r="22" spans="1:11" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="22" t="s">
+        <v>13</v>
+      </c>
+      <c r="B22" s="21" t="s">
+        <v>14</v>
+      </c>
+      <c r="C22" s="31" t="s">
+        <v>20</v>
+      </c>
+      <c r="D22" s="31"/>
+      <c r="E22" s="31" t="s">
+        <v>19</v>
+      </c>
+      <c r="F22" s="33"/>
+      <c r="G22" s="16"/>
+    </row>
+    <row r="23" spans="1:11" ht="24.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="23" t="s">
+        <v>21</v>
+      </c>
+      <c r="B23" s="20" t="s">
+        <v>15</v>
+      </c>
+      <c r="C23" s="32" t="s">
+        <v>22</v>
+      </c>
+      <c r="D23" s="32"/>
+      <c r="E23" s="32" t="s">
+        <v>23</v>
+      </c>
+      <c r="F23" s="34"/>
+      <c r="G23" s="10"/>
+      <c r="H23" s="11"/>
+      <c r="I23" s="11"/>
+      <c r="J23" s="11"/>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="G24" s="12"/>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A25" s="28" t="s">
         <v>4</v>
       </c>
-      <c r="H22" s="7"/>
-      <c r="I22" s="7"/>
-      <c r="J22" s="7"/>
-      <c r="K22" s="7"/>
-    </row>
-    <row r="23" spans="1:11" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="22" t="s">
+      <c r="B25" s="28"/>
+      <c r="C25" s="28"/>
+      <c r="D25" s="28"/>
+      <c r="E25" s="28"/>
+      <c r="F25" s="28"/>
+      <c r="G25" s="17"/>
+      <c r="H25" s="17"/>
+      <c r="I25" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="B23" s="23" t="s">
-        <v>6</v>
-      </c>
-      <c r="C23" s="23" t="s">
+    </row>
+    <row r="44" spans="1:10" ht="36" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="45" spans="1:10" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A45" s="11"/>
+      <c r="B45" s="11"/>
+      <c r="C45" s="11"/>
+      <c r="D45" s="11"/>
+      <c r="E45" s="11"/>
+      <c r="F45" s="11"/>
+      <c r="G45" s="11"/>
+      <c r="H45" s="11"/>
+      <c r="I45" s="11"/>
+      <c r="J45" s="11"/>
+    </row>
+    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A46" s="13" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A47" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D23" s="23" t="s">
-        <v>8</v>
-      </c>
-      <c r="E23" s="23" t="s">
+      <c r="B47" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="F23" s="24" t="s">
-        <v>10</v>
-      </c>
-      <c r="G23" s="16"/>
-      <c r="H23" s="17"/>
-      <c r="I23" s="17"/>
-      <c r="J23" s="17"/>
-      <c r="K23" s="17"/>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="F24" s="18"/>
-      <c r="G24" s="18"/>
-    </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="C25" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="I25" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="44" spans="1:11" ht="36" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="45" spans="1:11" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="17"/>
-      <c r="B45" s="17"/>
-      <c r="C45" s="17"/>
-      <c r="D45" s="17"/>
-      <c r="E45" s="17"/>
-      <c r="F45" s="17"/>
-      <c r="G45" s="17"/>
-      <c r="H45" s="17"/>
-      <c r="I45" s="17"/>
-      <c r="J45" s="17"/>
-      <c r="K45" s="17"/>
-    </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A46" s="20" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A47" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B47" s="20" t="s">
-        <v>17</v>
-      </c>
     </row>
   </sheetData>
+  <mergeCells count="14">
+    <mergeCell ref="A25:F25"/>
+    <mergeCell ref="I20:K20"/>
+    <mergeCell ref="C22:D22"/>
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="E22:F22"/>
+    <mergeCell ref="E23:F23"/>
+    <mergeCell ref="C21:D21"/>
+    <mergeCell ref="E21:F21"/>
+    <mergeCell ref="G8:J8"/>
+    <mergeCell ref="G7:J7"/>
+    <mergeCell ref="G10:J10"/>
+    <mergeCell ref="G11:J11"/>
+    <mergeCell ref="G12:J12"/>
+    <mergeCell ref="G9:J9"/>
+  </mergeCells>
   <pageMargins left="0.23622047244094491" right="0.23622047244094491" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
   <drawing r:id="rId2"/>

</xml_diff>